<commit_message>
Move molecular_subtype to Clinical_Features.xlsx column (per-subject)
- read_mol_subtypes() reads 'molecular_subtype' column from the spreadsheet,
  allowing each subject to have a different subtype in one run
- --mol_subtype CLI flag becomes an optional fallback (applied to all subjects
  when the column is absent); leaving a cell blank or 'unknown' skips DL-M2
  for that subject only
- step3_dlm2 and step4b now iterate per-subject instead of batch-predicting
  a single shared subtype
- example/Clinical_Features.xlsx updated with molecular_subtype column
  (SUBJ001=KIAA1549_BRAF, SUBJ002=BRAF_V600E, SUBJ003=NF1)
- README and example/README updated accordingly
</commit_message>
<xml_diff>
--- a/example/Clinical_Features.xlsx
+++ b/example/Clinical_Features.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,11 @@
           <t>radiation</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>molecular_subtype</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -509,6 +514,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>KIAA1549_BRAF</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -549,6 +559,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>BRAF_V600E</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -587,6 +602,11 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NF1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Separate age at diagnosis from age at imaging for the molecular model
DL-M1 is trained on age at the imaging event; the molecular model that
feeds DL-M2 is trained on age at DIAGNOSIS. The pipeline was feeding
age_at_event_days to both.

These are not interchangeable. Across the 294 subjects common to both
cohorts, 21 (7%) have differing values -- by up to 4342 days (~12 years).
Substituting one for the other shifts the DL-M2 score by up to 0.40 and
flips at least one patient's risk group (C4074252: Low -> High).

- Clinical_Features.xlsx gains an optional age_at_diagnosis_days column,
  used by the molecular model; DL-M1 continues to use age_at_event_days
- Falls back to age_at_event_days with a one-time warning when the new
  column is absent, so existing spreadsheets keep working
- README documents why both columns exist; example file carries both

Regression after change: molecular 493/493 exact, DL-M2 294/294 exact,
risk group 294/294 agree.
</commit_message>
<xml_diff>
--- a/example/Clinical_Features.xlsx
+++ b/example/Clinical_Features.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,30 +446,35 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>age_at_diagnosis_days</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>consolidated_tumor_locations</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>cancer_predisposition</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>extent_of_tumor_resection</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>chemotherapy</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>radiation</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>molecular_subtype</t>
         </is>
@@ -489,32 +494,35 @@
       <c r="C2" t="n">
         <v>2920</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>2920</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Cerebellar</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>None documented</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Gross/Near total resection</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>KIAA1549_BRAF</t>
         </is>
@@ -534,32 +542,35 @@
       <c r="C3" t="n">
         <v>4380</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4380</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Suprasellar</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>None documented</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Biopsy only</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>BRAF_V600E</t>
         </is>
@@ -579,32 +590,35 @@
       <c r="C4" t="n">
         <v>1825</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="n">
+        <v>1825</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Brain Stem</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Neurofibromatosis, Type 1 (NF-1)</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Partial resection</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>NF1</t>
         </is>

</xml_diff>

<commit_message>
Use a single age column for both DL-M1 and the molecular model
Reverts the two-column split from the previous commit. At inference time
a patient has one age, so requiring two age fields invites transcription
error for no benefit. Both models now read age_at_event_days (age at
diagnosis); each still applies its own StandardScaler, fit on its own
training cohort.

The 7% train-time discrepancy between the two source spreadsheets is an
artifact of the retrospective cohort assembly, not something to propagate
into the inference API. Published per-patient results are unaffected --
they came from the reference run, which read each model's own source.

README documents that one age feeds both models and that the differing
scalers are expected. Regression: molecular 493/493 exact, DL-M2 294/294
exact, risk group 294/294 agree.
</commit_message>
<xml_diff>
--- a/example/Clinical_Features.xlsx
+++ b/example/Clinical_Features.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,35 +446,30 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>age_at_diagnosis_days</t>
+          <t>consolidated_tumor_locations</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>consolidated_tumor_locations</t>
+          <t>cancer_predisposition</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>cancer_predisposition</t>
+          <t>extent_of_tumor_resection</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>extent_of_tumor_resection</t>
+          <t>chemotherapy</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>chemotherapy</t>
+          <t>radiation</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>radiation</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>molecular_subtype</t>
         </is>
@@ -494,22 +489,24 @@
       <c r="C2" t="n">
         <v>2920</v>
       </c>
-      <c r="D2" t="n">
-        <v>2920</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Cerebellar</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Cerebellar</t>
+          <t>None documented</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>None documented</t>
+          <t>Gross/Near total resection</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Gross/Near total resection</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -518,11 +515,6 @@
         </is>
       </c>
       <c r="I2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
         <is>
           <t>KIAA1549_BRAF</t>
         </is>
@@ -542,35 +534,32 @@
       <c r="C3" t="n">
         <v>4380</v>
       </c>
-      <c r="D3" t="n">
-        <v>4380</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Suprasellar</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Suprasellar</t>
+          <t>None documented</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>None documented</t>
+          <t>Biopsy only</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Biopsy only</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
         <is>
           <t>BRAF_V600E</t>
         </is>
@@ -590,35 +579,32 @@
       <c r="C4" t="n">
         <v>1825</v>
       </c>
-      <c r="D4" t="n">
-        <v>1825</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Brain Stem</t>
+        </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Brain Stem</t>
+          <t>Neurofibromatosis, Type 1 (NF-1)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Neurofibromatosis, Type 1 (NF-1)</t>
+          <t>Partial resection</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Partial resection</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
         <is>
           <t>NF1</t>
         </is>

</xml_diff>